<commit_message>
Online Reporting and some delay fixes in Prod Verification Script
</commit_message>
<xml_diff>
--- a/KatalonData/BWPBootstrapData/BWPACHData.xlsx
+++ b/KatalonData/BWPBootstrapData/BWPACHData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3167" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3387" uniqueCount="678">
   <si>
     <t>Result</t>
   </si>
@@ -1778,6 +1778,336 @@
   </si>
   <si>
     <t>Tue Jun 09 20:07:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 01:59:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:01:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:04:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:05:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:05:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:06:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:07:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:08:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:14:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:15:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:15:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:16:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:17:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:18:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:19:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:20:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:21:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:22:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:22:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:23:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:24:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:25:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:26:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:27:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:28:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:29:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:30:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:31:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:32:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:39:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:40:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:41:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:43:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:44:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:52:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:53:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:54:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:55:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:56:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:57:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:58:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 02:59:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:00:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:00:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:01:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:03:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:03:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:05:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:07:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:08:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:10:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:11:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:11:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:12:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:14:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:15:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:15:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:17:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:17:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:18:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:26:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:27:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:27:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:29:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:29:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:30:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:31:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:32:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:33:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:44:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:45:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:46:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:47:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:49:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:50:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:51:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:52:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:54:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:55:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:55:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:57:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:58:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 03:58:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:04:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:05:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:06:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:08:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:10:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:11:45 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:13:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:14:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:14:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:15:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:16:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:17:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:19:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:19:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:21:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:23:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:24:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:25:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:25:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:26:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:27:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:27:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:28:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 04:29:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 19:12:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 19:17:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 21 19:25:03 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -2116,7 +2446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
@@ -2167,11 +2497,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>533</v>
+      <c r="B2" t="s" s="0">
+        <v>677</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -2216,7 +2546,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84B2224-A06F-477C-8FF6-AF4C244AA0CE}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
@@ -2267,11 +2597,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>543</v>
+      <c r="B2" t="s" s="0">
+        <v>663</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -2311,7 +2641,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366B0B2-5D78-426C-AEBB-C29C53584E7F}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2359,11 +2689,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>549</v>
+      <c r="B2" t="s" s="0">
+        <v>669</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2403,7 +2733,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35ACE39D-499D-49B4-BFD2-CDDE6D0F8728}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2451,11 +2781,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>541</v>
+      <c r="B2" t="s" s="0">
+        <v>660</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2495,7 +2825,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29FACBAA-68A5-4A1D-8E32-A4AA8B032AE1}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2543,11 +2873,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>502</v>
+      <c r="B2" t="s" s="0">
+        <v>621</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2587,7 +2917,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924F2B64-1D9A-415C-B98F-EB7A7BAB8DD9}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2635,11 +2965,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>510</v>
+      <c r="B2" t="s" s="0">
+        <v>628</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2679,7 +3009,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A084124A-76B7-4B99-A6AD-5B2A169F9B8A}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2727,11 +3057,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>511</v>
+      <c r="B2" t="s" s="0">
+        <v>629</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2771,7 +3101,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0332CA16-31EB-4917-9936-860E79D3523B}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2819,11 +3149,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>512</v>
+      <c r="B2" t="s" s="0">
+        <v>630</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2863,7 +3193,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1E53DD-391D-45C7-A26E-A3CBEF12F623}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2911,11 +3241,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>513</v>
+      <c r="B2" t="s" s="0">
+        <v>631</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2955,7 +3285,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65676D18-4455-410B-8CF0-024536C3D41C}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3003,11 +3333,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>514</v>
+      <c r="B2" t="s" s="0">
+        <v>632</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3047,7 +3377,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06203600-C68B-4759-93E3-003ACDDD00D9}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3095,11 +3425,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>515</v>
+      <c r="B2" t="s" s="0">
+        <v>633</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3139,7 +3469,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188BD99A-2280-478C-8415-3AF3B8D2E566}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3187,11 +3517,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>535</v>
+      <c r="B2" t="s" s="0">
+        <v>657</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -3233,7 +3563,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{044EB785-1D8B-4520-A589-98FB5248CE3B}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3281,11 +3611,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>516</v>
+      <c r="B2" t="s" s="0">
+        <v>634</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3325,7 +3655,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAB2259B-110A-4E54-AAE6-DB14B9EB5171}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3373,11 +3703,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>517</v>
+      <c r="B2" t="s" s="0">
+        <v>635</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3417,7 +3747,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE735932-BE48-4F0B-B6E0-1AACE863DBE6}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3465,11 +3795,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>518</v>
+      <c r="B2" t="s" s="0">
+        <v>636</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3509,7 +3839,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FDA41C-A48E-4DF7-9F3C-4EA15B85EA24}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3557,11 +3887,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>522</v>
+      <c r="B2" t="s" s="0">
+        <v>642</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3601,7 +3931,7 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6653DFE2-5232-47EC-B0F1-E3DFB6BF3E7A}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3649,11 +3979,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>524</v>
+      <c r="B2" t="s" s="0">
+        <v>644</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3693,7 +4023,7 @@
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C026E37F-098F-42E5-92AB-1E317624CC4D}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -3741,11 +4071,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>523</v>
+      <c r="B2" t="s" s="0">
+        <v>643</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3785,7 +4115,7 @@
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE16B14-240B-4522-A71A-377E72FADE1F}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
@@ -3874,7 +4204,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E5825C-6EEF-49AA-9880-B92945E2442C}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
@@ -3963,7 +4293,7 @@
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B10A84-4465-4F3C-AB05-F2529380B3EA}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
@@ -4054,7 +4384,7 @@
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD262109-C636-4152-9E03-BF0F49D8C917}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
@@ -4105,10 +4435,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>71</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -4151,7 +4481,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CB3A07-E958-4D14-B792-C4C5D72CD8EA}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -4199,11 +4529,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>501</v>
+      <c r="B2" t="s" s="0">
+        <v>620</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4243,7 +4573,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FBEB25C-002A-46ED-B528-BBFB127AD6B5}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
@@ -4294,10 +4624,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>76</v>
       </c>
       <c r="C2" s="3"/>
@@ -4338,7 +4668,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A3C05C-8E29-42C3-A89E-8ED671B7BB31}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
@@ -4389,10 +4719,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>76</v>
       </c>
       <c r="C2" s="3"/>
@@ -4433,7 +4763,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB610E4-D8A9-4F86-99AA-691BCAA68B9C}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -4481,11 +4811,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>525</v>
+      <c r="B2" t="s" s="0">
+        <v>645</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4525,7 +4855,7 @@
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3C025A-C3F4-4ABF-9C60-AA1DCCB0BC50}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -4573,11 +4903,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>526</v>
+      <c r="B2" t="s" s="0">
+        <v>646</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4617,7 +4947,7 @@
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A067396-2824-448F-9289-4B8D3E2041FE}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -4665,11 +4995,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>527</v>
+      <c r="B2" t="s" s="0">
+        <v>647</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4709,7 +5039,7 @@
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AECE1F9-32F0-48E5-B835-168A7EF42FA8}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -4757,11 +5087,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>528</v>
+      <c r="B2" t="s" s="0">
+        <v>648</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4801,7 +5131,7 @@
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AEB8BAF-D441-4510-B01C-E6A2F0E35EEA}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -4849,11 +5179,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>529</v>
+      <c r="B2" t="s" s="0">
+        <v>649</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4893,7 +5223,7 @@
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4CCB5A6-D07A-4BC3-BD3B-767113A862D2}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -4941,11 +5271,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>530</v>
+      <c r="B2" t="s" s="0">
+        <v>650</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4985,7 +5315,7 @@
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F93338-8AAA-4B19-8B9D-4771302FEFC0}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="17.21875" collapsed="true"/>
@@ -5036,11 +5366,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>548</v>
+      <c r="B2" t="s" s="0">
+        <v>668</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>25</v>
@@ -5082,7 +5412,7 @@
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC6E653-D4E4-4FCF-8BD0-11D4CBABA3A9}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
@@ -5133,11 +5463,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>565</v>
+      <c r="B2" t="s" s="0">
+        <v>667</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5177,7 +5507,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893E9D9E-A65A-420C-985F-4AFBCEBD5458}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5225,11 +5555,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>531</v>
+      <c r="B2" t="s" s="0">
+        <v>651</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5269,7 +5599,7 @@
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF98BAE0-3DBA-4724-A623-84E06EAD3F5D}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
@@ -5320,11 +5650,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>520</v>
+      <c r="B2" t="s" s="0">
+        <v>638</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5364,7 +5694,7 @@
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CD5E31-F635-4FC0-9668-1419F01D6942}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5412,11 +5742,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>508</v>
+      <c r="B2" t="s" s="0">
+        <v>626</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5456,7 +5786,7 @@
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD2F0AE-7828-442C-A2B3-21D0EBE7331D}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
@@ -5507,11 +5837,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>505</v>
+      <c r="B2" t="s" s="0">
+        <v>623</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5551,7 +5881,7 @@
 
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62E2C147-58C7-49F8-940A-3E37DE049451}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5599,11 +5929,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>553</v>
+      <c r="B2" t="s" s="0">
+        <v>675</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5643,7 +5973,7 @@
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC79200-E4B3-4160-86F6-78B06F6EA2C0}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5691,11 +6021,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>564</v>
+      <c r="B2" t="s" s="0">
+        <v>674</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5735,7 +6065,7 @@
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026E9C75-7C58-441D-91D6-25552A135B0A}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5783,11 +6113,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>550</v>
+      <c r="B2" t="s" s="0">
+        <v>670</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5827,7 +6157,7 @@
 
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D307F9B9-84A6-4F70-AF5F-E09C0B70177D}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5875,11 +6205,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>566</v>
+      <c r="B2" t="s" s="0">
+        <v>672</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5919,7 +6249,7 @@
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CED210A-15BA-4154-A75C-369A0BF113DA}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5967,11 +6297,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>567</v>
+      <c r="B2" t="s" s="0">
+        <v>673</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>26</v>
@@ -6013,7 +6343,7 @@
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13CCEC20-911A-47BC-B790-0438DD3BE26D}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -6061,11 +6391,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>521</v>
+      <c r="B2" t="s" s="0">
+        <v>641</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -6105,7 +6435,7 @@
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE927C8-204D-43C3-9530-F9F77785B40B}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -6153,11 +6483,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>506</v>
+      <c r="B2" t="s" s="0">
+        <v>624</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -6197,7 +6527,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F88BD42D-CC7A-48FA-8796-B59D2B587379}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -6245,11 +6575,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>540</v>
+      <c r="B2" t="s" s="0">
+        <v>659</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -6289,7 +6619,7 @@
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAABB2E9-54E4-4860-85B4-28F35D889E47}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -6337,11 +6667,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>509</v>
+      <c r="B2" t="s" s="0">
+        <v>627</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -6381,7 +6711,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B65B44A-04F0-4B2C-962C-6C956F0737B9}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
@@ -6432,11 +6762,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>504</v>
+      <c r="B2" t="s" s="0">
+        <v>622</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -6476,7 +6806,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A462096B-4AF9-4B81-B6B6-00EE8E7EF270}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -6524,11 +6854,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>507</v>
+      <c r="B2" t="s" s="0">
+        <v>625</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -6568,7 +6898,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04E9BD2B-9C3A-4D4A-991E-C6044AE36784}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
@@ -6619,11 +6949,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>519</v>
+      <c r="B2" t="s" s="0">
+        <v>637</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -6663,7 +6993,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A723C119-E528-48BF-99DE-522307C92146}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="19.0" collapsed="true"/>
@@ -6714,11 +7044,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>539</v>
+      <c r="B2" t="s" s="0">
+        <v>658</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>

</xml_diff>